<commit_message>
showcase re-recorded on the P&L variance (PLG-20): new transcript, filed outputs, images; 8/8 seals verify; variance.json hashes to the test constant; README timing and golden description
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/showcase/may-26/filed/Variance Report - May-26 SIGNED KL.xlsx
+++ b/showcase/may-26/filed/Variance Report - May-26 SIGNED KL.xlsx
@@ -54,11 +54,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -432,6 +433,8 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,7 +447,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Actual per trial balance; budget per Budget FY26 - by line. Flag threshold ±100. Caldergate Distribution Group Ltd - Confidential. Fictitious data (demo estate).</t>
+          <t>Actual per trial balance; budget per Budget FY26 - by line. Variance = actual - budget; F/A = effect on profit. Flag threshold ±100. Caldergate Distribution Group Ltd - Confidential. Fictitious data (demo estate).</t>
         </is>
       </c>
     </row>
@@ -483,6 +486,11 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>F/A</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Flag</t>
         </is>
       </c>
@@ -507,6 +515,11 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>FLAG</t>
         </is>
       </c>
@@ -531,6 +544,11 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>FLAG</t>
         </is>
       </c>
@@ -553,195 +571,334 @@
       <c r="E7" t="n">
         <v>1.9</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Cost of goods sold</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>15843</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>15599</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>244</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>FLAG</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>21063</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>20753</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>310</v>
+      </c>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Warehouse &amp; Logistics</t>
+          <t>Cost of goods sold</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>1661</v>
+        <v>15843</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1663</v>
+        <v>15599</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-2</v>
+        <v>244</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1</v>
+        <v>1.6</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FLAG</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Sales &amp; Account Management</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>1257</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>1230</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="E10" t="n">
-        <v>2.2</v>
-      </c>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Gross margin</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>5220</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>5154</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Procurement &amp; Merchandising</t>
+          <t>Warehouse &amp; Logistics</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>597</v>
+        <v>1661</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>586</v>
+        <v>1663</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>11</v>
+        <v>-2</v>
       </c>
       <c r="E11" t="n">
-        <v>1.9</v>
+        <v>-0.1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IT &amp; Digital</t>
+          <t>Sales &amp; Account Management</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>521</v>
+        <v>1257</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>519</v>
+        <v>1230</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4</v>
+        <v>2.2</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>General &amp; Administrative</t>
+          <t>Procurement &amp; Merchandising</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>796</v>
+        <v>597</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>807</v>
+        <v>586</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-11</v>
+        <v>11</v>
       </c>
       <c r="E13" t="n">
-        <v>-1.4</v>
+        <v>1.9</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Depreciation &amp; amortisation</t>
+          <t>IT &amp; Digital</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>400</v>
+        <v>521</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>400</v>
+        <v>519</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>0.4</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Interest expense, net</t>
+          <t>General &amp; Administrative</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>132</v>
+        <v>796</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>132</v>
+        <v>807</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0</v>
+        <v>-11</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>-1.4</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Taxation</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>-36</v>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>-36</v>
-      </c>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Total operating expenses</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>4832</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>4805</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>42234</v>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>41689</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>545</v>
-      </c>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>388</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>349</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; amortisation</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Interest expense, net</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>132</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>132</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Taxation</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>-36</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>-36</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Net result</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>-108</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>-183</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -754,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -767,25 +924,19 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Actual 8,343 against budget 8,216, a variance of +127.0 (+1.5%), £'000, MTD May-26. Driver not evidenced in the documents: Commercial Director to comment. (Sources checked: close notes, trial balance, budget workbook; none states a cause.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>## Industrial Consumables &amp; Packaging</t>
-        </is>
-      </c>
-    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Revenue was 8,343 against a budget of 8,216, a favourable variance of +127.0 (+1.5%). Driver not evidenced in the documents: Commercial Director to comment. The only comparative on file, the April-26 v2 FINAL report, describes April's adverse variance on this line as the mirror of March's NHS call-off timing. It says nothing about May, so no cause is given for May's variance. Source checked: `99 Board/Monthly Report - Apr-26 (v2 FINAL).pdf`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Actual 8,464 against budget 8,361, a variance of +103.0 (+1.2%), £'000, MTD May-26. Driver not evidenced in the documents: Commercial Director to comment. (Sources checked: close notes, trial balance, budget workbook; none states a cause.)</t>
+          <t>## Industrial Consumables &amp; Packaging</t>
         </is>
       </c>
     </row>
@@ -793,14 +944,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Revenue was 8,464 against a budget of 8,361, a favourable variance of +103.0 (+1.2%). Driver not evidenced in the documents: Commercial Director to comment. April was restated for a £620k cut-off correction on this line (orders invoiced ahead of despatch), per the April-26 v2 FINAL report. No document links that correction to May's variance, so none is claimed. Source checked: `99 Board/Monthly Report - Apr-26 (v2 FINAL).pdf`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>## Cost of goods sold</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Actual 15,843 against budget 15,599, a variance of +244.0 (+1.6%), £'000, MTD May-26. Driver not evidenced in the documents: Head of Procurement to comment. (Sources checked: close notes, trial balance, budget workbook; none states a cause.)</t>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cost of goods sold was 15,843 against a budget of 15,599, an adverse variance of +244.0 (+1.6%). Driver not evidenced in the documents: Head of Procurement to comment. No document in the close folder attributes the cost to volume, price or mix. Sources checked: the close notes and `99 Board/Monthly Report - Apr-26 (v2 FINAL).pdf`.</t>
         </is>
       </c>
     </row>

</xml_diff>